<commit_message>
feat: fixed constraint lessonConflict (no instructor teaches to lessons at the same time)
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/output/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/output/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="110">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -75,64 +75,67 @@
     <t>MWF 11:00 - 12:00</t>
   </si>
   <si>
+    <t>MWF 14:00 - 15:00</t>
+  </si>
+  <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>De Moura Canaan, Rodrigo</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
+    <t>MWF 07:00 - 08:00</t>
+  </si>
+  <si>
+    <t>csc481</t>
+  </si>
+  <si>
     <t>MWF 12:00 - 13:00</t>
   </si>
   <si>
-    <t>De Moura Canaan, Rodrigo</t>
-  </si>
-  <si>
-    <t>csc480</t>
-  </si>
-  <si>
-    <t>MWF 07:00 - 08:00</t>
-  </si>
-  <si>
-    <t>csc481</t>
+    <t>Dekhtyar, Alexander M.</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>Eckhardt, Christian</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>TR 15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>TR 16:30 - 18:00</t>
+  </si>
+  <si>
+    <t>Einakian, Sussan</t>
+  </si>
+  <si>
+    <t>csc101</t>
   </si>
   <si>
     <t>MWF 13:00 - 14:00</t>
   </si>
   <si>
-    <t>Dekhtyar, Alexander M.</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>Eckhardt, Christian</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>TR 15:00 - 16:30</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>MWF 14:00 - 15:00</t>
-  </si>
-  <si>
-    <t>255</t>
+    <t>232A</t>
   </si>
   <si>
     <t>Frishberg, Daniel</t>
@@ -165,150 +168,153 @@
     <t>csc378</t>
   </si>
   <si>
+    <t>Hristov, Borislav</t>
+  </si>
+  <si>
+    <t>csc448</t>
+  </si>
+  <si>
     <t>MWF 17:00 - 18:00</t>
   </si>
   <si>
-    <t>Hristov, Borislav</t>
-  </si>
-  <si>
-    <t>csc448</t>
+    <t>Hsu, Silas</t>
+  </si>
+  <si>
+    <t>csc437</t>
   </si>
   <si>
     <t>MWF 18:00 - 19:00</t>
   </si>
   <si>
-    <t>Hsu, Silas</t>
-  </si>
-  <si>
-    <t>csc437</t>
+    <t>Jones, Brian Thomas</t>
+  </si>
+  <si>
+    <t>csc232</t>
+  </si>
+  <si>
+    <t>MW 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>MW 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>MTWR 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>MTWR 12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>Kalathas, Paris</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>Kazerouni, Ayaan</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>Keen, Aaron</t>
+  </si>
+  <si>
+    <t>Khan, Fahim Hasan</t>
+  </si>
+  <si>
+    <t>csc471</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 19:30</t>
+  </si>
+  <si>
+    <t>Klingenberg, Bernhard J.</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>Kubiak, Kenneth E.</t>
+  </si>
+  <si>
+    <t>csc307</t>
+  </si>
+  <si>
+    <t>192-333</t>
+  </si>
+  <si>
+    <t>Lindqvist, Ulf Erik</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>Mukherjee, Joydeep</t>
+  </si>
+  <si>
+    <t>csc410</t>
+  </si>
+  <si>
+    <t>Nico, Phillip L.</t>
+  </si>
+  <si>
+    <t>csc453</t>
+  </si>
+  <si>
+    <t>Pantoja, Maria</t>
+  </si>
+  <si>
+    <t>csc569</t>
+  </si>
+  <si>
+    <t>TR 18:30 - 20:00</t>
+  </si>
+  <si>
+    <t>TR 20:00 - 21:30</t>
+  </si>
+  <si>
+    <t>Peterson, Zachary N.J.</t>
+  </si>
+  <si>
+    <t>Pierce, Lucas Shane</t>
+  </si>
+  <si>
+    <t>csc466</t>
+  </si>
+  <si>
+    <t>20-127</t>
+  </si>
+  <si>
+    <t>Rathi, Anita</t>
+  </si>
+  <si>
+    <t>Rivera, Vanessa</t>
+  </si>
+  <si>
+    <t>Rwebangira, Mugizi Robert</t>
+  </si>
+  <si>
+    <t>csc566</t>
+  </si>
+  <si>
+    <t>csc349</t>
+  </si>
+  <si>
+    <t>TR 16:00 - 17:30</t>
+  </si>
+  <si>
+    <t>TR 17:30 - 19:00</t>
+  </si>
+  <si>
+    <t>Schmitt, Paul</t>
+  </si>
+  <si>
+    <t>Siu, Christopher E.</t>
   </si>
   <si>
     <t>MWF 19:00 - 20:00</t>
   </si>
   <si>
-    <t>Jones, Brian Thomas</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>TR 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>TR 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>MTWR 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>MTWR 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>Kalathas, Paris</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>Kazerouni, Ayaan</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>Keen, Aaron</t>
-  </si>
-  <si>
-    <t>Khan, Fahim Hasan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>TR 18:00 - 19:30</t>
-  </si>
-  <si>
-    <t>Klingenberg, Bernhard J.</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>Kubiak, Kenneth E.</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>Lindqvist, Ulf Erik</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>Mukherjee, Joydeep</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>Nico, Phillip L.</t>
-  </si>
-  <si>
-    <t>csc453</t>
-  </si>
-  <si>
-    <t>Pantoja, Maria</t>
-  </si>
-  <si>
-    <t>csc569</t>
-  </si>
-  <si>
-    <t>TR 18:30 - 20:00</t>
-  </si>
-  <si>
-    <t>TR 20:00 - 21:30</t>
-  </si>
-  <si>
-    <t>Peterson, Zachary N.J.</t>
-  </si>
-  <si>
-    <t>Pierce, Lucas Shane</t>
-  </si>
-  <si>
-    <t>csc466</t>
-  </si>
-  <si>
-    <t>Rathi, Anita</t>
-  </si>
-  <si>
-    <t>301</t>
-  </si>
-  <si>
-    <t>Rivera, Vanessa</t>
-  </si>
-  <si>
-    <t>Rwebangira, Mugizi Robert</t>
-  </si>
-  <si>
-    <t>csc566</t>
-  </si>
-  <si>
-    <t>csc349</t>
-  </si>
-  <si>
-    <t>Schmitt, Paul</t>
-  </si>
-  <si>
-    <t>Siu, Christopher E.</t>
-  </si>
-  <si>
     <t>Stanchev, Lubomir Petrov</t>
   </si>
   <si>
@@ -318,12 +324,6 @@
     <t>Teo, Ka Yaw</t>
   </si>
   <si>
-    <t>TR 16:00 - 17:30</t>
-  </si>
-  <si>
-    <t>TR 17:30 - 19:00</t>
-  </si>
-  <si>
     <t>Ventura, Jonathan Daniel</t>
   </si>
   <si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>csc321</t>
+  </si>
+  <si>
+    <t>257</t>
   </si>
   <si>
     <t>Zielke, Christopher Patrick</t>
@@ -509,18 +512,18 @@
         <v>8</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" t="b" s="0">
         <v>1</v>
@@ -529,7 +532,7 @@
         <v>8</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>9</v>
@@ -537,10 +540,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" t="b" s="0">
         <v>1</v>
@@ -549,18 +552,18 @@
         <v>8</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" t="b" s="0">
         <v>1</v>
@@ -569,7 +572,7 @@
         <v>8</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>29</v>
@@ -609,18 +612,18 @@
         <v>8</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
@@ -629,15 +632,15 @@
         <v>8</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>7</v>
@@ -646,18 +649,18 @@
         <v>1</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>28</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>7</v>
@@ -666,61 +669,61 @@
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C17" t="b" s="0">
         <v>1</v>
@@ -729,10 +732,10 @@
         <v>8</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +752,7 @@
         <v>8</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s" s="0">
         <v>53</v>
@@ -800,19 +803,19 @@
         <v>57</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22">
@@ -820,19 +823,19 @@
         <v>57</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>61</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
@@ -840,19 +843,19 @@
         <v>57</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C23" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E23" t="s" s="0">
         <v>62</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
@@ -866,7 +869,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E24" t="s" s="0">
         <v>10</v>
@@ -886,13 +889,13 @@
         <v>1</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26">
@@ -906,13 +909,13 @@
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>28</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27">
@@ -926,13 +929,13 @@
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>19</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28">
@@ -949,24 +952,24 @@
         <v>8</v>
       </c>
       <c r="E28" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="F28" t="s" s="0">
         <v>70</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>71</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B29" t="s" s="0">
         <v>72</v>
       </c>
-      <c r="B29" t="s" s="0">
-        <v>73</v>
-      </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>13</v>
@@ -977,16 +980,16 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B30" t="s" s="0">
         <v>72</v>
       </c>
-      <c r="B30" t="s" s="0">
-        <v>73</v>
-      </c>
       <c r="C30" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E30" t="s" s="0">
         <v>32</v>
@@ -997,27 +1000,27 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="B31" t="s" s="0">
         <v>74</v>
       </c>
-      <c r="B31" t="s" s="0">
-        <v>75</v>
-      </c>
       <c r="C31" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="F31" t="s" s="0">
         <v>39</v>
-      </c>
-      <c r="E31" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="F31" t="s" s="0">
-        <v>25</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B32" t="s" s="0">
         <v>55</v>
@@ -1026,18 +1029,18 @@
         <v>1</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s" s="0">
         <v>55</v>
@@ -1046,13 +1049,13 @@
         <v>1</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34">
@@ -1066,13 +1069,13 @@
         <v>1</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35">
@@ -1086,7 +1089,7 @@
         <v>1</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>33</v>
@@ -1106,7 +1109,7 @@
         <v>1</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>13</v>
@@ -1117,36 +1120,36 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B37" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B37" t="s" s="0">
-        <v>82</v>
-      </c>
       <c r="C37" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B38" t="s" s="0">
-        <v>82</v>
-      </c>
       <c r="C38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>10</v>
@@ -1157,10 +1160,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="B39" t="s" s="0">
         <v>83</v>
-      </c>
-      <c r="B39" t="s" s="0">
-        <v>84</v>
       </c>
       <c r="C39" t="b" s="0">
         <v>1</v>
@@ -1169,24 +1172,24 @@
         <v>8</v>
       </c>
       <c r="E39" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F39" t="s" s="0">
         <v>85</v>
-      </c>
-      <c r="F39" t="s" s="0">
-        <v>86</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E40" t="s" s="0">
         <v>17</v>
@@ -1197,42 +1200,42 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="B41" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="B41" t="s" s="0">
-        <v>89</v>
-      </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E41" t="s" s="0">
         <v>19</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="B42" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="C42" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="C42" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D42" t="s" s="0">
-        <v>80</v>
-      </c>
       <c r="E42" t="s" s="0">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s" s="0">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="43">
@@ -1240,19 +1243,19 @@
         <v>90</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E43" t="s" s="0">
         <v>29</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44">
@@ -1260,13 +1263,13 @@
         <v>90</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E44" t="s" s="0">
         <v>9</v>
@@ -1286,7 +1289,7 @@
         <v>1</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>13</v>
@@ -1297,7 +1300,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B46" t="s" s="0">
         <v>31</v>
@@ -1306,18 +1309,18 @@
         <v>1</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s" s="0">
         <v>31</v>
@@ -1326,18 +1329,18 @@
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B48" t="s" s="0">
         <v>31</v>
@@ -1346,98 +1349,98 @@
         <v>1</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B49" t="s" s="0">
         <v>93</v>
-      </c>
-      <c r="B49" t="s" s="0">
-        <v>94</v>
       </c>
       <c r="C49" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E49" t="s" s="0">
         <v>61</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B50" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="C50" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D50" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E50" t="s" s="0">
         <v>95</v>
       </c>
-      <c r="C50" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D50" t="s" s="0">
-        <v>39</v>
-      </c>
-      <c r="E50" t="s" s="0">
-        <v>50</v>
-      </c>
       <c r="F50" t="s" s="0">
-        <v>53</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B53" t="s" s="0">
         <v>31</v>
@@ -1446,73 +1449,73 @@
         <v>1</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>56</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>101</v>
+        <v>32</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>102</v>
+        <v>33</v>
       </c>
     </row>
     <row r="57">
@@ -1520,19 +1523,19 @@
         <v>103</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58">
@@ -1546,13 +1549,13 @@
         <v>0</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59">
@@ -1566,13 +1569,13 @@
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="60">
@@ -1586,30 +1589,30 @@
         <v>1</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F61" t="s" s="0">
         <v>9</v>
@@ -1617,42 +1620,42 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>29</v>
+        <v>53</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="C63" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D63" t="s" s="0">
         <v>107</v>
       </c>
-      <c r="B63" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="C63" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D63" t="s" s="0">
-        <v>91</v>
-      </c>
       <c r="E63" t="s" s="0">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>